<commit_message>
data(cmr): richer bundled cmr-example.xlsx with realistic coverage spread (0.9.3)
The bundled CMR example had a flat ~95% coverage across every district, so
figures built from it couldn't tell a "which district is behind target"
story. Adjust the per-district `#rbtrt_treated` / `#schtrt_treated` values so
coverage spans ~62-99% (Kampala 99, Mbarara 62, Soroti 87 for oncho; Kampala
88, Mbarara 99 for sch). Structure, sheets, field codes and row counts are
unchanged; only the treated values differ. Purely demonstration data.

Follow-on to the atlantis training sandbox (#263/#264): makes the CMR-guide
and training figures actually informative. Bump to 0.9.3 + NEWS.
</commit_message>
<xml_diff>
--- a/inst/extdata/cmr-example.xlsx
+++ b/inst/extdata/cmr-example.xlsx
@@ -447,7 +447,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>11400</t>
+          <t>11880</t>
         </is>
       </c>
     </row>
@@ -479,7 +479,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>7600</t>
+          <t>4960</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>5800</t>
+          <t>5220</t>
         </is>
       </c>
     </row>
@@ -617,7 +617,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>4800</t>
+          <t>4400</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2900</t>
+          <t>2970</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(cmr): richer bundled cmr-example.xlsx with realistic coverage spread (0.9.3) (#265)
The bundled CMR example had a flat ~95% coverage across every district, so
figures built from it couldn't tell a "which district is behind target"
story. Adjust the per-district `#rbtrt_treated` / `#schtrt_treated` values so
coverage spans ~62-99% (Kampala 99, Mbarara 62, Soroti 87 for oncho; Kampala
88, Mbarara 99 for sch). Structure, sheets, field codes and row counts are
unchanged; only the treated values differ. Purely demonstration data.

Follow-on to the atlantis training sandbox (#263/#264): makes the CMR-guide
and training figures actually informative. Bump to 0.9.3 + NEWS.
</commit_message>
<xml_diff>
--- a/inst/extdata/cmr-example.xlsx
+++ b/inst/extdata/cmr-example.xlsx
@@ -447,7 +447,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>11400</t>
+          <t>11880</t>
         </is>
       </c>
     </row>
@@ -479,7 +479,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>7600</t>
+          <t>4960</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>5800</t>
+          <t>5220</t>
         </is>
       </c>
     </row>
@@ -617,7 +617,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>4800</t>
+          <t>4400</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2900</t>
+          <t>2970</t>
         </is>
       </c>
     </row>

</xml_diff>